<commit_message>
update FinalReport.docx and AILogs
</commit_message>
<xml_diff>
--- a/ai_logs/HoangNam_AILogs.xlsx
+++ b/ai_logs/HoangNam_AILogs.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21000" windowHeight="9180" firstSheet="1" activeTab="3"/>
+    <workbookView windowWidth="23040" windowHeight="9708" firstSheet="1" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="1. Metadata &amp; Summary" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="280">
   <si>
     <t>AI AUDIT LOG - METADATA &amp; SUMMARY</t>
   </si>
@@ -450,6 +450,51 @@
     <t>011</t>
   </si>
   <si>
+    <t>Code Design</t>
+  </si>
+  <si>
+    <t>Admin View Integration</t>
+  </si>
+  <si>
+    <t>Cần một phần Admin riêng để quản lý nhân sự, chi nhánh và doanh thu trong hệ thống nhà thuốc.</t>
+  </si>
+  <si>
+    <t>Thiết kế AdminView và AdminController để quản lý pharmacist, branch và báo cáo doanh thu, tách riêng khỏi luồng của pharmacist.</t>
+  </si>
+  <si>
+    <t>Tạo menu Admin riêng với CRUD staff, CRUD branch có bảo vệ khi xóa, và báo cáo doanh thu theo 30 ngày / toàn thời gian.</t>
+  </si>
+  <si>
+    <t>Mình xác nhận rằng trách nhiệm của Admin khác hoàn toàn với phần quản lý thuốc của pharmacist. Vì vậy mình tách logic admin ra controller/view riêng để rõ ràng và dễ bảo trì hơn.</t>
+  </si>
+  <si>
+    <t>AdminController.java; AdminView.java</t>
+  </si>
+  <si>
+    <t>012</t>
+  </si>
+  <si>
+    <t>Verification</t>
+  </si>
+  <si>
+    <t>Main Routing / Role Handling</t>
+  </si>
+  <si>
+    <t>Cần tích hợp Admin view vào luồng chạy chính mà không làm hỏng đăng nhập hiện có.</t>
+  </si>
+  <si>
+    <t>Gắn menu Admin vào MainView và đảm bảo routing theo role vẫn hoạt động sau khi thêm controller mới.</t>
+  </si>
+  <si>
+    <t>Cập nhật wiring để user ADMIN mở AdminView, còn STAFF vẫn dùng menu pharmacist.</t>
+  </si>
+  <si>
+    <t>Mình kiểm tra lại phân quyền sau refactor và giữ nguyên đăng nhập bằng số điện thoại. Luồng admin được nạp qua dependency injection nên giảm coupling.</t>
+  </si>
+  <si>
+    <t>Main.java; MainView.java; User.java</t>
+  </si>
+  <si>
     <t>HALLUCINATION DETECTION LOG (BẮT BUỘC)</t>
   </si>
   <si>
@@ -639,9 +684,6 @@
     <t>Bỏ input thừa ở menu chính, chuyển việc nhập branch ID vào từng chức năng con</t>
   </si>
   <si>
-    <t>012</t>
-  </si>
-  <si>
     <t>Scope Confusion</t>
   </si>
   <si>
@@ -657,6 +699,42 @@
     <t>Cập nhật hàm report nhận branch ID và lọc dữ liệu theo chi nhánh tương ứng</t>
   </si>
   <si>
+    <t>013</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Oversimplification</t>
+  </si>
+  <si>
+    <t>AI cho rằng chỉ cần thêm một menu mới ở tầng UI là đủ để có Admin view.</t>
+  </si>
+  <si>
+    <t>Thực tế còn cần controller riêng, ràng buộc xóa branch, và logic tổng hợp doanh thu, không chỉ là một màn hình menu.</t>
+  </si>
+  <si>
+    <t>So sánh gợi ý của AI với kế hoạch triển khai và trách nhiệm thực tế của Admin trong codebase.</t>
+  </si>
+  <si>
+    <t>Tạo AdminController/AdminView, thêm bảo vệ khi quản lý branch, và giữ logic doanh thu ngoài UI layer.</t>
+  </si>
+  <si>
+    <t>014</t>
+  </si>
+  <si>
+    <t>Context Misunderstanding</t>
+  </si>
+  <si>
+    <t>AI ban đầu trộn lẫn trách nhiệm của Admin với phần quản lý thuốc.</t>
+  </si>
+  <si>
+    <t>Admin trong project này quản lý staff, branch và doanh thu; còn CRUD thuốc thuộc về MedicineController riêng.</t>
+  </si>
+  <si>
+    <t>Kiểm tra lại cấu trúc menu và ranh giới giữa các controller sau refactor.</t>
+  </si>
+  <si>
+    <t>Tách MedicineController khỏi StockController và giữ phần Admin chỉ tập trung vào nghiệp vụ quản trị.</t>
+  </si>
+  <si>
     <t>HALLUCINATION TYPES REFERENCE:</t>
   </si>
   <si>
@@ -703,9 +781,6 @@
   </si>
   <si>
     <t>Old API syntax, deprecated methods</t>
-  </si>
-  <si>
-    <t>Context Misunderstanding</t>
   </si>
   <si>
     <t>AI không hiểu đúng bối cảnh</t>
@@ -2522,23 +2597,53 @@
       <c r="A14" s="26" t="s">
         <v>133</v>
       </c>
-      <c r="B14" s="15"/>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="15"/>
+      <c r="B14" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="F14" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="G14" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="H14" s="15" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="15" ht="80" customHeight="1" spans="1:8">
-      <c r="A15" s="15"/>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
+      <c r="A15" s="26" t="s">
+        <v>141</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="F15" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="G15" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="H15" s="15" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="16" ht="80" customHeight="1" spans="1:8">
       <c r="A16" s="15"/>
@@ -2673,32 +2778,32 @@
   <sheetData>
     <row r="1" ht="21" spans="1:6">
       <c r="A1" s="16" t="s">
-        <v>134</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="17" t="s">
-        <v>135</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3" ht="40" customHeight="1" spans="1:6">
       <c r="A3" s="4" t="s">
-        <v>136</v>
+        <v>151</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>138</v>
+        <v>153</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>139</v>
+        <v>154</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
     </row>
     <row r="4" ht="60" customHeight="1" spans="1:6">
@@ -2706,19 +2811,19 @@
         <v>56</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>142</v>
+        <v>157</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>143</v>
+        <v>158</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>144</v>
+        <v>159</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>145</v>
+        <v>160</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>146</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5" ht="57.6" spans="1:6">
@@ -2726,19 +2831,19 @@
         <v>64</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>147</v>
+        <v>162</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>148</v>
+        <v>163</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>149</v>
+        <v>164</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>150</v>
+        <v>165</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>151</v>
+        <v>166</v>
       </c>
     </row>
     <row r="6" ht="60" customHeight="1" spans="1:6">
@@ -2746,19 +2851,19 @@
         <v>72</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>152</v>
+        <v>167</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>153</v>
+        <v>168</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>154</v>
+        <v>169</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>155</v>
+        <v>170</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>156</v>
+        <v>171</v>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1" spans="1:6">
@@ -2766,19 +2871,19 @@
         <v>80</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>157</v>
+        <v>172</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>158</v>
+        <v>173</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>159</v>
+        <v>174</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>160</v>
+        <v>175</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>161</v>
+        <v>176</v>
       </c>
     </row>
     <row r="8" ht="60" customHeight="1" spans="1:6">
@@ -2786,19 +2891,19 @@
         <v>88</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>162</v>
+        <v>177</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>163</v>
+        <v>178</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>164</v>
+        <v>179</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>165</v>
+        <v>180</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>166</v>
+        <v>181</v>
       </c>
     </row>
     <row r="9" ht="60" customHeight="1" spans="1:6">
@@ -2806,19 +2911,19 @@
         <v>96</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>168</v>
+        <v>183</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>169</v>
+        <v>184</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="10" ht="60" customHeight="1" spans="1:6">
@@ -2826,19 +2931,19 @@
         <v>104</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>172</v>
+        <v>187</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>173</v>
+        <v>188</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>174</v>
+        <v>189</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>176</v>
+        <v>191</v>
       </c>
     </row>
     <row r="11" ht="60" customHeight="1" spans="1:6">
@@ -2846,19 +2951,19 @@
         <v>111</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>177</v>
+        <v>192</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>178</v>
+        <v>193</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>179</v>
+        <v>194</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>180</v>
+        <v>195</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>181</v>
+        <v>196</v>
       </c>
     </row>
     <row r="12" ht="60" customHeight="1" spans="1:6">
@@ -2866,19 +2971,19 @@
         <v>118</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>182</v>
+        <v>197</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>183</v>
+        <v>198</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>184</v>
+        <v>199</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>185</v>
+        <v>200</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>186</v>
+        <v>201</v>
       </c>
     </row>
     <row r="13" ht="60" customHeight="1" spans="1:6">
@@ -2886,19 +2991,19 @@
         <v>125</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>187</v>
+        <v>202</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>188</v>
+        <v>203</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>189</v>
+        <v>204</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>190</v>
+        <v>205</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>191</v>
+        <v>206</v>
       </c>
     </row>
     <row r="14" ht="60" customHeight="1" spans="1:6">
@@ -2906,56 +3011,80 @@
         <v>133</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>194</v>
+        <v>209</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>195</v>
+        <v>210</v>
       </c>
       <c r="F14" s="15" t="s">
-        <v>196</v>
+        <v>211</v>
       </c>
     </row>
     <row r="15" ht="60" customHeight="1" spans="1:6">
       <c r="A15" s="26" t="s">
-        <v>197</v>
+        <v>141</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>198</v>
+        <v>212</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>199</v>
+        <v>213</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>200</v>
+        <v>214</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>201</v>
+        <v>215</v>
       </c>
       <c r="F15" s="15" t="s">
-        <v>202</v>
+        <v>216</v>
       </c>
     </row>
     <row r="16" ht="60" customHeight="1" spans="1:6">
-      <c r="A16" s="15"/>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
+      <c r="A16" s="26" t="s">
+        <v>217</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>218</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>219</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>220</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>221</v>
+      </c>
+      <c r="F16" s="15" t="s">
+        <v>222</v>
+      </c>
     </row>
     <row r="17" ht="60" customHeight="1" spans="1:6">
-      <c r="A17" s="15"/>
-      <c r="B17" s="15"/>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
+      <c r="A17" s="26" t="s">
+        <v>223</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>224</v>
+      </c>
+      <c r="C17" s="15" t="s">
+        <v>225</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>226</v>
+      </c>
+      <c r="E17" s="15" t="s">
+        <v>227</v>
+      </c>
+      <c r="F17" s="15" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="18" ht="60" customHeight="1" spans="1:6">
       <c r="A18" s="15"/>
@@ -3015,73 +3144,73 @@
     </row>
     <row r="30" ht="18" spans="1:6">
       <c r="A30" s="3" t="s">
-        <v>203</v>
+        <v>229</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="13" t="s">
-        <v>204</v>
+        <v>230</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>205</v>
+        <v>231</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>206</v>
+        <v>232</v>
       </c>
     </row>
     <row r="32" ht="28.8" spans="1:6">
       <c r="A32" s="15" t="s">
-        <v>207</v>
+        <v>233</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>208</v>
+        <v>234</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>209</v>
+        <v>235</v>
       </c>
     </row>
     <row r="33" ht="28.8" spans="1:3">
       <c r="A33" s="15" t="s">
-        <v>210</v>
+        <v>236</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>211</v>
+        <v>237</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>212</v>
+        <v>238</v>
       </c>
     </row>
     <row r="34" ht="28.8" spans="1:3">
       <c r="A34" s="15" t="s">
-        <v>213</v>
+        <v>239</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>214</v>
+        <v>240</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>215</v>
+        <v>241</v>
       </c>
     </row>
     <row r="35" ht="28.8" spans="1:3">
       <c r="A35" s="15" t="s">
-        <v>216</v>
+        <v>242</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>217</v>
+        <v>243</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>218</v>
+        <v>244</v>
       </c>
     </row>
     <row r="36" ht="43.2" spans="1:3">
       <c r="A36" s="15" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>220</v>
+        <v>245</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>221</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -3108,42 +3237,42 @@
   <sheetData>
     <row r="1" ht="21" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>222</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
-        <v>223</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4" ht="18" spans="1:4">
       <c r="A4" s="3" t="s">
-        <v>224</v>
+        <v>249</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="4" t="s">
-        <v>225</v>
+        <v>250</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>226</v>
+        <v>251</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>227</v>
+        <v>252</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>228</v>
+        <v>253</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="6" t="s">
-        <v>229</v>
+        <v>254</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>230</v>
+        <v>255</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>231</v>
+        <v>256</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>36</v>
@@ -3151,13 +3280,13 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="6" t="s">
-        <v>232</v>
+        <v>257</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>233</v>
+        <v>258</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>231</v>
+        <v>256</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>36</v>
@@ -3165,13 +3294,13 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="6" t="s">
-        <v>234</v>
+        <v>259</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>235</v>
+        <v>260</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>231</v>
+        <v>256</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>36</v>
@@ -3179,13 +3308,13 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="6" t="s">
-        <v>236</v>
+        <v>261</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>237</v>
+        <v>262</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>231</v>
+        <v>256</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>36</v>
@@ -3193,13 +3322,13 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="6" t="s">
-        <v>238</v>
+        <v>263</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>239</v>
+        <v>264</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>231</v>
+        <v>256</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>36</v>
@@ -3207,32 +3336,32 @@
     </row>
     <row r="12" ht="18" spans="1:4">
       <c r="A12" s="3" t="s">
-        <v>240</v>
+        <v>265</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="4" t="s">
-        <v>225</v>
+        <v>250</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>226</v>
+        <v>251</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>227</v>
+        <v>252</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>241</v>
+        <v>266</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="6" t="s">
-        <v>229</v>
+        <v>254</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>242</v>
+        <v>267</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>231</v>
+        <v>256</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>36</v>
@@ -3240,13 +3369,13 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="6" t="s">
-        <v>232</v>
+        <v>257</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>243</v>
+        <v>268</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>231</v>
+        <v>256</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>36</v>
@@ -3254,13 +3383,13 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="6" t="s">
-        <v>234</v>
+        <v>259</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>244</v>
+        <v>269</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>231</v>
+        <v>256</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>36</v>
@@ -3268,13 +3397,13 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="6" t="s">
-        <v>236</v>
+        <v>261</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>245</v>
+        <v>270</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>231</v>
+        <v>256</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>36</v>
@@ -3282,13 +3411,13 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="6" t="s">
-        <v>238</v>
+        <v>263</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>246</v>
+        <v>271</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>231</v>
+        <v>256</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>36</v>
@@ -3296,27 +3425,27 @@
     </row>
     <row r="20" ht="15.6" spans="1:4">
       <c r="A20" s="9" t="s">
-        <v>247</v>
+        <v>272</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="10" t="s">
-        <v>248</v>
+        <v>273</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="10" t="s">
-        <v>249</v>
+        <v>274</v>
       </c>
     </row>
     <row r="25" ht="18" spans="1:4">
       <c r="A25" s="3" t="s">
-        <v>250</v>
+        <v>275</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="11" t="s">
-        <v>251</v>
+        <v>276</v>
       </c>
     </row>
     <row r="27" ht="43.2" spans="1:4">
@@ -3324,13 +3453,13 @@
         <v>48</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>252</v>
+        <v>277</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>253</v>
+        <v>278</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>254</v>
+        <v>279</v>
       </c>
     </row>
     <row r="28" spans="1:4">

</xml_diff>